<commit_message>
IPL Dashboard created in this commit
</commit_message>
<xml_diff>
--- a/vlookup-hlookup.xlsx
+++ b/vlookup-hlookup.xlsx
@@ -1,34 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASDC11\Desktop\smit\Data_Analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smit\OneDrive\Desktop\Data Analyst\Data_Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C6FC9DA-5D5D-4C1F-90D1-978B9FD4F9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E709F3-0227-4E28-93BC-69695A4A382B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{174E6243-5B42-4101-9076-EB3932145E51}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{174E6243-5B42-4101-9076-EB3932145E51}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -119,7 +110,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -227,11 +218,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -257,61 +263,21 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FF3D444D"/>
-        </left>
-        <right style="medium">
-          <color rgb="FF3D444D"/>
-        </right>
-        <top style="medium">
-          <color rgb="FF3D444D"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FF3D444D"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -345,6 +311,173 @@
         <top style="medium">
           <color rgb="FF3D444D"/>
         </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="medium">
           <color rgb="FF3D444D"/>
         </bottom>
@@ -385,132 +518,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF3D444D"/>
-        </left>
-        <right style="medium">
-          <color rgb="FF3D444D"/>
-        </right>
-        <top style="medium">
-          <color rgb="FF3D444D"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FF3D444D"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="medium">
-          <color rgb="FF3D444D"/>
-        </right>
-        <top style="medium">
-          <color rgb="FF3D444D"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FF3D444D"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FF3D444D"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color rgb="FF3D444D"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FF3D444D"/>
-        </left>
-        <right style="medium">
-          <color rgb="FF3D444D"/>
-        </right>
-        <top style="medium">
-          <color rgb="FF3D444D"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FF3D444D"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -525,13 +532,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F52B1F6F-6508-4D98-B90D-3D38B985C208}" name="Table1" displayName="Table1" ref="A3:D8" totalsRowShown="0" headerRowDxfId="2" dataDxfId="3" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F52B1F6F-6508-4D98-B90D-3D38B985C208}" name="Table1" displayName="Table1" ref="A3:D8" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A3:D8" xr:uid="{F52B1F6F-6508-4D98-B90D-3D38B985C208}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DD1843F0-2016-481C-AF25-99F282FD751C}" name="Roll No" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{11D536A0-080C-494C-B9FF-0273892CEA5F}" name="Student Name" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{6F0792CF-11B9-4B4F-97C5-4B76ECBFA425}" name="Marks" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{83DD8E2F-E33F-4416-93D5-81717CD143AE}" name="Result" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{DD1843F0-2016-481C-AF25-99F282FD751C}" name="Roll No" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{11D536A0-080C-494C-B9FF-0273892CEA5F}" name="Student Name" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{6F0792CF-11B9-4B4F-97C5-4B76ECBFA425}" name="Marks" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{83DD8E2F-E33F-4416-93D5-81717CD143AE}" name="Result" dataDxfId="0">
       <calculatedColumnFormula>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -836,17 +843,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDFA88DF-2307-4BDF-8B1D-60018EBC1791}">
-  <dimension ref="A3:N27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A3:N12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>8</v>
       </c>
@@ -860,7 +867,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -874,13 +881,13 @@
         <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-    </row>
-    <row r="5" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+    </row>
+    <row r="5" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -894,11 +901,11 @@
         <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
         <v>Fail</v>
       </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-    </row>
-    <row r="6" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+    </row>
+    <row r="6" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -912,11 +919,11 @@
         <f>IF(Table1[[#This Row],[Marks]]&gt;=40,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-    </row>
-    <row r="7" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+    </row>
+    <row r="7" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>4</v>
       </c>
@@ -931,7 +938,7 @@
         <v>Pass</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>5</v>
       </c>
@@ -946,124 +953,21 @@
         <v>Fail</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C11" t="s">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C12" t="s">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C12" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12" s="12" t="str">
         <f>VLOOKUP(C12,Table1[[#All],[Student Name]:[Result]],3,0)</f>
         <v>Fail</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="2">
-        <v>1</v>
-      </c>
-      <c r="C20" s="2">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2">
-        <v>3</v>
-      </c>
-      <c r="E20" s="2">
-        <v>4</v>
-      </c>
-      <c r="F20" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="2">
-        <v>82</v>
-      </c>
-      <c r="C22" s="2">
-        <v>35</v>
-      </c>
-      <c r="D22" s="2">
-        <v>62</v>
-      </c>
-      <c r="E22" s="2">
-        <v>40</v>
-      </c>
-      <c r="F22" s="2">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B23" s="2" t="str">
-        <f>IF(B22&gt;=40,"Pass","Fail")</f>
-        <v>Pass</v>
-      </c>
-      <c r="C23" s="2" t="str">
-        <f t="shared" ref="C23:F23" si="0">IF(C22&gt;=40,"Pass","Fail")</f>
-        <v>Fail</v>
-      </c>
-      <c r="D23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Pass</v>
-      </c>
-      <c r="E23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Pass</v>
-      </c>
-      <c r="F23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Fail</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B27">
-        <v>4</v>
-      </c>
-      <c r="D27" t="str">
-        <f>HLOOKUP(B27,A20:F23,4,0)</f>
-        <v>Pass</v>
       </c>
     </row>
   </sheetData>
@@ -1082,4 +986,117 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02066C4E-D271-4EC9-862F-EFBD2672405A}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:6" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="39" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2">
+        <v>82</v>
+      </c>
+      <c r="C4" s="2">
+        <v>35</v>
+      </c>
+      <c r="D4" s="2">
+        <v>62</v>
+      </c>
+      <c r="E4" s="2">
+        <v>40</v>
+      </c>
+      <c r="F4" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="19.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <f>IF(B4&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <f>IF(C4&gt;=40,"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <f>IF(D4&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <f>IF(E4&gt;=40,"Pass","Fail")</f>
+        <v>Pass</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <f>IF(F4&gt;=40,"Pass","Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E7" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E8" s="12">
+        <v>5</v>
+      </c>
+      <c r="F8" s="12" t="str">
+        <f>HLOOKUP(E8,Sheet2!A2:F5,4,0)</f>
+        <v>Fail</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>